<commit_message>
progress: 25 village workbooks (randomwalk-TRX50-WS 2026-10-09T11:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Rettambedu_13.426632_80.16966.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Rettambedu_13.426632_80.16966.xlsx
@@ -1130,11 +1130,6 @@
           <t>150</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1142,11 +1137,6 @@
           <t>151</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1154,11 +1144,6 @@
           <t>152</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>10A, 10B, 11, 12A1, 12A2, 12B1, 12B2, 13, 1A, 1B, 2B1, 2B2, 3A, 4, 5, 6A, 6B, 7A1, 7A2, 7B1, 7B2, 8A1, 8A2, 8B1, 8B2, 9</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1166,11 +1151,6 @@
           <t>153</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2A, 2B, 3, 4, 5A, 5B, 6A1, 6A2, 6B, 6C, 6D, 7</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1178,11 +1158,6 @@
           <t>154</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1190,11 +1165,6 @@
           <t>155</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1202,11 +1172,6 @@
           <t>156</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1214,11 +1179,6 @@
           <t>157</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1226,11 +1186,6 @@
           <t>158</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B1A, 2B2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1238,11 +1193,6 @@
           <t>159</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1250,11 +1200,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B, 6</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1262,11 +1207,6 @@
           <t>160</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1274,11 +1214,6 @@
           <t>161</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1286,11 +1221,6 @@
           <t>162</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1298,11 +1228,6 @@
           <t>163</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A1, 3A2, 3B, 4A, 4B1, 4B2</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1310,11 +1235,6 @@
           <t>164</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1322,11 +1242,6 @@
           <t>165</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4A, 4B, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1334,11 +1249,6 @@
           <t>166</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 2A, 2B, 3A, 3B, 4, 5, 6A, 6B1, 6B2, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1346,11 +1256,6 @@
           <t>167</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7A, 7B, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1358,11 +1263,6 @@
           <t>168</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A, 3B, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1370,11 +1270,6 @@
           <t>169</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1382,11 +1277,6 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1394,11 +1284,6 @@
           <t>170</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2B1A, 2B1B, 2B1C, 2B2, 2B3, 2B4</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1406,11 +1291,6 @@
           <t>171</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1418,11 +1298,6 @@
           <t>172</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1430,11 +1305,6 @@
           <t>173</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B1, 2B2, 3, 4, 5A, 5B</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1442,11 +1312,6 @@
           <t>174</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6A, 6B, 7</t>
-        </is>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1454,11 +1319,6 @@
           <t>175</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1466,11 +1326,6 @@
           <t>176</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1478,11 +1333,6 @@
           <t>177</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1490,11 +1340,6 @@
           <t>178</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 3C, 4A, 4B, 5</t>
-        </is>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1502,11 +1347,6 @@
           <t>179</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1514,11 +1354,6 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1526,11 +1361,6 @@
           <t>180</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1538,11 +1368,6 @@
           <t>181</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1550,11 +1375,6 @@
           <t>182</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1562,11 +1382,6 @@
           <t>183</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1574,11 +1389,6 @@
           <t>184</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3</t>
-        </is>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1586,11 +1396,6 @@
           <t>185</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1598,11 +1403,6 @@
           <t>186</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1610,11 +1410,6 @@
           <t>187</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1622,11 +1417,6 @@
           <t>188</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1634,11 +1424,6 @@
           <t>189</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2A1, 2A2, 2B, 3</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1646,11 +1431,6 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1658,11 +1438,6 @@
           <t>190</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6A, 6B, 6C</t>
-        </is>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1670,11 +1445,6 @@
           <t>191</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1682,11 +1452,6 @@
           <t>192</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1694,11 +1459,6 @@
           <t>193</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1706,11 +1466,6 @@
           <t>194</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5, 6, 7A, 7B, 7C, 8</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1718,11 +1473,6 @@
           <t>195</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1730,11 +1480,6 @@
           <t>196</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1742,11 +1487,6 @@
           <t>197</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1754,11 +1494,6 @@
           <t>198</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1766,11 +1501,6 @@
           <t>199</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A1A1, 2B, 2C, 2D, 2E, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 4A, 5A1A, 5B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1778,11 +1508,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1790,11 +1515,6 @@
           <t>20</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1802,11 +1522,6 @@
           <t>200</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B1, 3B2, 3B3, 3B4, 3B5, 4A1A1, 4A2, 4A3, 4B, 4C, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1814,11 +1529,6 @@
           <t>201</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3A, 3B1A1A, 3B1B, 3B2, 3C, 3D, 3E, 3F, 3G, 3H, 3I, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1826,11 +1536,6 @@
           <t>202</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1838,11 +1543,6 @@
           <t>203</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1850,11 +1550,6 @@
           <t>204</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1862,11 +1557,6 @@
           <t>205</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 2</t>
-        </is>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1874,11 +1564,6 @@
           <t>206</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1886,11 +1571,6 @@
           <t>207</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1898,11 +1578,6 @@
           <t>208</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1910,11 +1585,6 @@
           <t>209</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1922,11 +1592,6 @@
           <t>21</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1934,11 +1599,6 @@
           <t>210</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1946,11 +1606,6 @@
           <t>211</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1958,11 +1613,6 @@
           <t>212</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1970,11 +1620,6 @@
           <t>213</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1982,11 +1627,6 @@
           <t>214</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1994,11 +1634,6 @@
           <t>215</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2006,11 +1641,6 @@
           <t>216</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2018,11 +1648,6 @@
           <t>217</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2030,11 +1655,6 @@
           <t>218</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2042,11 +1662,6 @@
           <t>219</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -2054,11 +1669,6 @@
           <t>22</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2066,11 +1676,6 @@
           <t>220</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 3A, 3B, 3C, 3D</t>
-        </is>
-      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2078,11 +1683,6 @@
           <t>221</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -2090,11 +1690,6 @@
           <t>222</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2102,11 +1697,6 @@
           <t>223</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2114,11 +1704,6 @@
           <t>224</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2126,11 +1711,6 @@
           <t>225</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 2, 20, 21, 22, 3A, 4, 5A, 5B, 6A1A, 6A1B, 6A1C, 6A1D, 6A2, 6B, 7A, 7B, 8A1A, 8B, 8C, 8D, 8E, 8F, 9A, 9B, 9C1, 9C2</t>
-        </is>
-      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -2138,11 +1718,6 @@
           <t>226</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2150,11 +1725,6 @@
           <t>227</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2162,11 +1732,6 @@
           <t>228</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2174,11 +1739,6 @@
           <t>229</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2186,11 +1746,6 @@
           <t>23</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2198,11 +1753,6 @@
           <t>230</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>1, 10, 2A, 2B, 3A, 3B, 4A1, 4A2, 4A3, 4A4, 4A5, 4B1, 4B2, 4B3A, 4B3B1, 4B3B2, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2210,11 +1760,6 @@
           <t>231</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2222,11 +1767,6 @@
           <t>232</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7A, 7B</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2234,11 +1774,6 @@
           <t>233</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2246,11 +1781,6 @@
           <t>234</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2258,11 +1788,6 @@
           <t>235</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2270,11 +1795,6 @@
           <t>236</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2282,11 +1802,6 @@
           <t>237</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2294,11 +1809,6 @@
           <t>238</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2306,11 +1816,6 @@
           <t>239</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A, 3B, 4A, 4B</t>
-        </is>
-      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2318,11 +1823,6 @@
           <t>24</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B1, 4B2</t>
-        </is>
-      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2330,11 +1830,6 @@
           <t>240</t>
         </is>
       </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2342,11 +1837,6 @@
           <t>241</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2354,11 +1844,6 @@
           <t>242</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2366,11 +1851,6 @@
           <t>243</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2378,11 +1858,6 @@
           <t>244</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2390,11 +1865,6 @@
           <t>245</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2402,11 +1872,6 @@
           <t>246</t>
         </is>
       </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B</t>
-        </is>
-      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2414,11 +1879,6 @@
           <t>247</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2426,11 +1886,6 @@
           <t>248</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2438,11 +1893,6 @@
           <t>249</t>
         </is>
       </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4A, 4B, 4C, 4D, 5A, 5B</t>
-        </is>
-      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2450,11 +1900,6 @@
           <t>25</t>
         </is>
       </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2462,11 +1907,6 @@
           <t>250</t>
         </is>
       </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2474,11 +1914,6 @@
           <t>251</t>
         </is>
       </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2486,11 +1921,6 @@
           <t>252</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2498,11 +1928,6 @@
           <t>253</t>
         </is>
       </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A, 12B, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2510,11 +1935,6 @@
           <t>254</t>
         </is>
       </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2522,11 +1942,6 @@
           <t>255</t>
         </is>
       </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2A1, 2A2, 2B1, 2B2, 2C1, 2C2, 3A1, 3A2, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2534,11 +1949,6 @@
           <t>256</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2546,11 +1956,6 @@
           <t>257</t>
         </is>
       </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>1, 10, 2A, 2B, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2558,11 +1963,6 @@
           <t>258</t>
         </is>
       </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2570,11 +1970,6 @@
           <t>259</t>
         </is>
       </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2582,11 +1977,6 @@
           <t>26</t>
         </is>
       </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A, 3B, 4</t>
-        </is>
-      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2594,11 +1984,6 @@
           <t>260</t>
         </is>
       </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2606,11 +1991,6 @@
           <t>261</t>
         </is>
       </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2618,11 +1998,6 @@
           <t>262</t>
         </is>
       </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 3</t>
-        </is>
-      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2630,11 +2005,6 @@
           <t>263</t>
         </is>
       </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B, 5C, 5D, 5E, 5F, 6</t>
-        </is>
-      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2642,11 +2012,6 @@
           <t>264</t>
         </is>
       </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2654,11 +2019,6 @@
           <t>265</t>
         </is>
       </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>-, 5A, 5C</t>
-        </is>
-      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2666,11 +2026,6 @@
           <t>266</t>
         </is>
       </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2678,11 +2033,6 @@
           <t>267</t>
         </is>
       </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2690,11 +2040,6 @@
           <t>268</t>
         </is>
       </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2702,11 +2047,6 @@
           <t>269</t>
         </is>
       </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2714,11 +2054,6 @@
           <t>27</t>
         </is>
       </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2726,11 +2061,6 @@
           <t>270</t>
         </is>
       </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2738,11 +2068,6 @@
           <t>271</t>
         </is>
       </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2750,11 +2075,6 @@
           <t>272</t>
         </is>
       </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2762,11 +2082,6 @@
           <t>273</t>
         </is>
       </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A1, 2A2, 2B, 3A1A, 3A1B, 3A2, 4, 5A1, 5A2, 5B, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2774,11 +2089,6 @@
           <t>274A</t>
         </is>
       </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2786,11 +2096,6 @@
           <t>274B</t>
         </is>
       </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2798,11 +2103,6 @@
           <t>274C</t>
         </is>
       </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2810,11 +2110,6 @@
           <t>275A</t>
         </is>
       </c>
-      <c r="B200" t="inlineStr">
-        <is>
-          <t>1A, A4</t>
-        </is>
-      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2822,11 +2117,6 @@
           <t>275B</t>
         </is>
       </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2834,11 +2124,6 @@
           <t>276</t>
         </is>
       </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2846,11 +2131,6 @@
           <t>277</t>
         </is>
       </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2858,11 +2138,6 @@
           <t>278</t>
         </is>
       </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2870,11 +2145,6 @@
           <t>279</t>
         </is>
       </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>10B1, 10B2, 11, 12, 1A2A7A10A, 1B, 2B, 3, 4, 5, 6, 7B1, 7B2, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2882,11 +2152,6 @@
           <t>28</t>
         </is>
       </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2894,11 +2159,6 @@
           <t>280</t>
         </is>
       </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2906,11 +2166,6 @@
           <t>281</t>
         </is>
       </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4, 5, 6A, 6B</t>
-        </is>
-      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2918,11 +2173,6 @@
           <t>282</t>
         </is>
       </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4A, 4B, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2930,11 +2180,6 @@
           <t>283</t>
         </is>
       </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2942,11 +2187,6 @@
           <t>284</t>
         </is>
       </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2954,11 +2194,6 @@
           <t>285</t>
         </is>
       </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2966,11 +2201,6 @@
           <t>286</t>
         </is>
       </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2978,11 +2208,6 @@
           <t>287</t>
         </is>
       </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2990,11 +2215,6 @@
           <t>288</t>
         </is>
       </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -3002,11 +2222,6 @@
           <t>289</t>
         </is>
       </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -3014,11 +2229,6 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -3026,11 +2236,6 @@
           <t>290</t>
         </is>
       </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -3038,11 +2243,6 @@
           <t>291</t>
         </is>
       </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -3050,11 +2250,6 @@
           <t>292</t>
         </is>
       </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 1B3, 2, 3, 4, 5B, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -3062,11 +2257,6 @@
           <t>293</t>
         </is>
       </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2B, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -3074,11 +2264,6 @@
           <t>294</t>
         </is>
       </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3B, 4, 5, 6B</t>
-        </is>
-      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -3086,11 +2271,6 @@
           <t>295</t>
         </is>
       </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5A, 5B, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -3098,11 +2278,6 @@
           <t>296</t>
         </is>
       </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -3110,11 +2285,6 @@
           <t>297</t>
         </is>
       </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 5</t>
-        </is>
-      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -3122,11 +2292,6 @@
           <t>298</t>
         </is>
       </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -3134,11 +2299,6 @@
           <t>299</t>
         </is>
       </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -3146,11 +2306,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -3158,11 +2313,6 @@
           <t>30</t>
         </is>
       </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -3170,11 +2320,6 @@
           <t>300</t>
         </is>
       </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -3182,11 +2327,6 @@
           <t>301</t>
         </is>
       </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -3194,11 +2334,6 @@
           <t>302</t>
         </is>
       </c>
-      <c r="B232" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -3206,11 +2341,6 @@
           <t>303</t>
         </is>
       </c>
-      <c r="B233" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -3218,11 +2348,6 @@
           <t>304</t>
         </is>
       </c>
-      <c r="B234" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 5A, 5B1, 5B2, 5C1, 5C2, 6</t>
-        </is>
-      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -3230,11 +2355,6 @@
           <t>305</t>
         </is>
       </c>
-      <c r="B235" t="inlineStr">
-        <is>
-          <t>1, 10, 2A, 2B, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -3242,11 +2362,6 @@
           <t>306</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -3254,11 +2369,6 @@
           <t>307</t>
         </is>
       </c>
-      <c r="B237" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -3266,11 +2376,6 @@
           <t>308</t>
         </is>
       </c>
-      <c r="B238" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -3278,11 +2383,6 @@
           <t>309</t>
         </is>
       </c>
-      <c r="B239" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -3290,11 +2390,6 @@
           <t>31</t>
         </is>
       </c>
-      <c r="B240" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -3302,11 +2397,6 @@
           <t>310</t>
         </is>
       </c>
-      <c r="B241" t="inlineStr">
-        <is>
-          <t>10, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -3314,11 +2404,6 @@
           <t>311</t>
         </is>
       </c>
-      <c r="B242" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -3326,11 +2411,6 @@
           <t>312</t>
         </is>
       </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -3338,11 +2418,6 @@
           <t>313</t>
         </is>
       </c>
-      <c r="B244" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -3350,11 +2425,6 @@
           <t>314</t>
         </is>
       </c>
-      <c r="B245" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -3362,11 +2432,6 @@
           <t>315</t>
         </is>
       </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -3374,11 +2439,6 @@
           <t>316</t>
         </is>
       </c>
-      <c r="B247" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22A, 22B, 23, 24, 25, 26, 27A1A, 27A1B, 27A1C, 27A2, 27B, 28A, 28B, 28C, 28D, 28E, 28F, 28G, 28H, 28I, 28J, 28K, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -3386,11 +2446,6 @@
           <t>317</t>
         </is>
       </c>
-      <c r="B248" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 2A, 2B, 2C, 2D, 2E</t>
-        </is>
-      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -3398,11 +2453,6 @@
           <t>318</t>
         </is>
       </c>
-      <c r="B249" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 2A, 2B, 2C, 2D, 2E, 2F, 2G1, 2G2</t>
-        </is>
-      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -3410,11 +2460,6 @@
           <t>319</t>
         </is>
       </c>
-      <c r="B250" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2, 3, 4, 5A, 5B, 6A, 6B, 6C, 6D, 6E</t>
-        </is>
-      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -3422,11 +2467,6 @@
           <t>32</t>
         </is>
       </c>
-      <c r="B251" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -3434,11 +2474,6 @@
           <t>320</t>
         </is>
       </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4A, 4B, 4C, 4D, 4E, 5, 6A, 6B</t>
-        </is>
-      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -3446,11 +2481,6 @@
           <t>321</t>
         </is>
       </c>
-      <c r="B253" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6A, 6B, 6C, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -3458,11 +2488,6 @@
           <t>322</t>
         </is>
       </c>
-      <c r="B254" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -3470,11 +2495,6 @@
           <t>323</t>
         </is>
       </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2A1A, 2A2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -3482,11 +2502,6 @@
           <t>324</t>
         </is>
       </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -3494,11 +2509,6 @@
           <t>325</t>
         </is>
       </c>
-      <c r="B257" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -3506,11 +2516,6 @@
           <t>326</t>
         </is>
       </c>
-      <c r="B258" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -3518,11 +2523,6 @@
           <t>327</t>
         </is>
       </c>
-      <c r="B259" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -3530,11 +2530,6 @@
           <t>328</t>
         </is>
       </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -3542,11 +2537,6 @@
           <t>329</t>
         </is>
       </c>
-      <c r="B261" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7A, 7B, 7C, 8</t>
-        </is>
-      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -3554,11 +2544,6 @@
           <t>33</t>
         </is>
       </c>
-      <c r="B262" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -3566,11 +2551,6 @@
           <t>330</t>
         </is>
       </c>
-      <c r="B263" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -3578,11 +2558,6 @@
           <t>331</t>
         </is>
       </c>
-      <c r="B264" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 5, 6, 7A, 7B, 8</t>
-        </is>
-      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -3590,11 +2565,6 @@
           <t>332</t>
         </is>
       </c>
-      <c r="B265" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 1A1A, 1A1B, 2A, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -3602,11 +2572,6 @@
           <t>333</t>
         </is>
       </c>
-      <c r="B266" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -3614,11 +2579,6 @@
           <t>334</t>
         </is>
       </c>
-      <c r="B267" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C</t>
-        </is>
-      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -3626,11 +2586,6 @@
           <t>335</t>
         </is>
       </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -3638,11 +2593,6 @@
           <t>336</t>
         </is>
       </c>
-      <c r="B269" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -3650,11 +2600,6 @@
           <t>337</t>
         </is>
       </c>
-      <c r="B270" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 3A, 3B, 4A, 4B, 5, 6A, 6B, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -3662,11 +2607,6 @@
           <t>338</t>
         </is>
       </c>
-      <c r="B271" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -3674,11 +2614,6 @@
           <t>339</t>
         </is>
       </c>
-      <c r="B272" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4, 5A, 5B, 6</t>
-        </is>
-      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -3686,11 +2621,6 @@
           <t>34</t>
         </is>
       </c>
-      <c r="B273" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -3698,11 +2628,6 @@
           <t>340</t>
         </is>
       </c>
-      <c r="B274" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -3710,11 +2635,6 @@
           <t>341</t>
         </is>
       </c>
-      <c r="B275" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -3722,11 +2642,6 @@
           <t>342</t>
         </is>
       </c>
-      <c r="B276" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B1, 2B2</t>
-        </is>
-      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -3734,11 +2649,6 @@
           <t>343</t>
         </is>
       </c>
-      <c r="B277" t="inlineStr">
-        <is>
-          <t>1, 10, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -3746,11 +2656,6 @@
           <t>344</t>
         </is>
       </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7A, 7B</t>
-        </is>
-      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -3758,11 +2663,6 @@
           <t>345</t>
         </is>
       </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 3A, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -3770,11 +2670,6 @@
           <t>346</t>
         </is>
       </c>
-      <c r="B280" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -3782,11 +2677,6 @@
           <t>347</t>
         </is>
       </c>
-      <c r="B281" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -3794,11 +2684,6 @@
           <t>348</t>
         </is>
       </c>
-      <c r="B282" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -3806,11 +2691,6 @@
           <t>349</t>
         </is>
       </c>
-      <c r="B283" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -3818,11 +2698,6 @@
           <t>35</t>
         </is>
       </c>
-      <c r="B284" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -3830,11 +2705,6 @@
           <t>350</t>
         </is>
       </c>
-      <c r="B285" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -3842,11 +2712,6 @@
           <t>351</t>
         </is>
       </c>
-      <c r="B286" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -3854,11 +2719,6 @@
           <t>352</t>
         </is>
       </c>
-      <c r="B287" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2</t>
-        </is>
-      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -3866,11 +2726,6 @@
           <t>353</t>
         </is>
       </c>
-      <c r="B288" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -3878,11 +2733,6 @@
           <t>354</t>
         </is>
       </c>
-      <c r="B289" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -3890,11 +2740,6 @@
           <t>355</t>
         </is>
       </c>
-      <c r="B290" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -3902,11 +2747,6 @@
           <t>356</t>
         </is>
       </c>
-      <c r="B291" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -3914,11 +2754,6 @@
           <t>357</t>
         </is>
       </c>
-      <c r="B292" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -3926,11 +2761,6 @@
           <t>358</t>
         </is>
       </c>
-      <c r="B293" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -3938,11 +2768,6 @@
           <t>359</t>
         </is>
       </c>
-      <c r="B294" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -3950,11 +2775,6 @@
           <t>36</t>
         </is>
       </c>
-      <c r="B295" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -3962,11 +2782,6 @@
           <t>360</t>
         </is>
       </c>
-      <c r="B296" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -3974,11 +2789,6 @@
           <t>361</t>
         </is>
       </c>
-      <c r="B297" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -3986,11 +2796,6 @@
           <t>362</t>
         </is>
       </c>
-      <c r="B298" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -3998,11 +2803,6 @@
           <t>363</t>
         </is>
       </c>
-      <c r="B299" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -4010,11 +2810,6 @@
           <t>364</t>
         </is>
       </c>
-      <c r="B300" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2, 3A, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -4022,11 +2817,6 @@
           <t>365</t>
         </is>
       </c>
-      <c r="B301" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -4034,11 +2824,6 @@
           <t>366</t>
         </is>
       </c>
-      <c r="B302" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14A, 14B1, 14B2, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 3, 4, 5, 6A, 6B, 7A, 7B, 7C, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -4046,11 +2831,6 @@
           <t>37</t>
         </is>
       </c>
-      <c r="B303" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -4058,11 +2838,6 @@
           <t>38</t>
         </is>
       </c>
-      <c r="B304" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -4070,11 +2845,6 @@
           <t>39</t>
         </is>
       </c>
-      <c r="B305" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A, 3B, 4</t>
-        </is>
-      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -4082,11 +2852,6 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B306" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A, 12B, 12C, 13A, 13B, 14, 15A, 15B, 16, 17, 18, 19, 2, 3, 4, 5A, 5B, 5C, 6A, 6B, 6C, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -4094,11 +2859,6 @@
           <t>40</t>
         </is>
       </c>
-      <c r="B307" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4A, 4B</t>
-        </is>
-      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -4106,11 +2866,6 @@
           <t>41</t>
         </is>
       </c>
-      <c r="B308" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B, 6A, 6B</t>
-        </is>
-      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -4118,11 +2873,6 @@
           <t>42</t>
         </is>
       </c>
-      <c r="B309" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B</t>
-        </is>
-      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -4130,11 +2880,6 @@
           <t>43</t>
         </is>
       </c>
-      <c r="B310" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -4142,11 +2887,6 @@
           <t>44</t>
         </is>
       </c>
-      <c r="B311" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -4154,11 +2894,6 @@
           <t>45</t>
         </is>
       </c>
-      <c r="B312" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -4166,11 +2901,6 @@
           <t>46</t>
         </is>
       </c>
-      <c r="B313" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -4178,11 +2908,6 @@
           <t>47</t>
         </is>
       </c>
-      <c r="B314" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -4190,11 +2915,6 @@
           <t>48</t>
         </is>
       </c>
-      <c r="B315" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -4202,11 +2922,6 @@
           <t>49</t>
         </is>
       </c>
-      <c r="B316" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -4214,11 +2929,6 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B317" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -4226,11 +2936,6 @@
           <t>50</t>
         </is>
       </c>
-      <c r="B318" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -4238,11 +2943,6 @@
           <t>51</t>
         </is>
       </c>
-      <c r="B319" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -4250,11 +2950,6 @@
           <t>52</t>
         </is>
       </c>
-      <c r="B320" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -4262,11 +2957,6 @@
           <t>53</t>
         </is>
       </c>
-      <c r="B321" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -4274,11 +2964,6 @@
           <t>54</t>
         </is>
       </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -4286,11 +2971,6 @@
           <t>55</t>
         </is>
       </c>
-      <c r="B323" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -4298,11 +2978,6 @@
           <t>56</t>
         </is>
       </c>
-      <c r="B324" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -4310,11 +2985,6 @@
           <t>57</t>
         </is>
       </c>
-      <c r="B325" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -4322,11 +2992,6 @@
           <t>58</t>
         </is>
       </c>
-      <c r="B326" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -4334,11 +2999,6 @@
           <t>59</t>
         </is>
       </c>
-      <c r="B327" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -4346,11 +3006,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B328" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -4358,11 +3013,6 @@
           <t>60</t>
         </is>
       </c>
-      <c r="B329" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -4370,11 +3020,6 @@
           <t>61</t>
         </is>
       </c>
-      <c r="B330" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -4382,11 +3027,6 @@
           <t>62</t>
         </is>
       </c>
-      <c r="B331" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -4394,11 +3034,6 @@
           <t>63</t>
         </is>
       </c>
-      <c r="B332" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -4406,11 +3041,6 @@
           <t>64</t>
         </is>
       </c>
-      <c r="B333" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4</t>
-        </is>
-      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -4418,11 +3048,6 @@
           <t>65</t>
         </is>
       </c>
-      <c r="B334" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2B, 3B, 4B, 5B</t>
-        </is>
-      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -4430,11 +3055,6 @@
           <t>66</t>
         </is>
       </c>
-      <c r="B335" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -4442,11 +3062,6 @@
           <t>67</t>
         </is>
       </c>
-      <c r="B336" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -4454,11 +3069,6 @@
           <t>68</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -4466,11 +3076,6 @@
           <t>69</t>
         </is>
       </c>
-      <c r="B338" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -4478,11 +3083,6 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B339" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -4490,11 +3090,6 @@
           <t>70</t>
         </is>
       </c>
-      <c r="B340" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -4502,11 +3097,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="B341" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -4514,11 +3104,6 @@
           <t>72</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -4526,11 +3111,6 @@
           <t>73</t>
         </is>
       </c>
-      <c r="B343" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -4538,11 +3118,6 @@
           <t>74</t>
         </is>
       </c>
-      <c r="B344" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -4550,11 +3125,6 @@
           <t>75</t>
         </is>
       </c>
-      <c r="B345" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -4562,11 +3132,6 @@
           <t>76</t>
         </is>
       </c>
-      <c r="B346" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 15C, 16, 17, 18A1, 18A2, 18B, 19A, 19B, 2, 20, 21A, 21B1, 21B2, 22, 23, 24, 25, 26, 27, 28, 3A, 3B, 4, 5A, 5B, 6A, 6B, 7A1, 7A2, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -4574,11 +3139,6 @@
           <t>77</t>
         </is>
       </c>
-      <c r="B347" t="inlineStr">
-        <is>
-          <t>1, 2A, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -4586,11 +3146,6 @@
           <t>78</t>
         </is>
       </c>
-      <c r="B348" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 3C</t>
-        </is>
-      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -4598,11 +3153,6 @@
           <t>79</t>
         </is>
       </c>
-      <c r="B349" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -4610,11 +3160,6 @@
           <t>8</t>
         </is>
       </c>
-      <c r="B350" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -4622,11 +3167,6 @@
           <t>80</t>
         </is>
       </c>
-      <c r="B351" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 5, 6A, 6B1, 6B2, 6B3, 7</t>
-        </is>
-      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -4634,11 +3174,6 @@
           <t>81</t>
         </is>
       </c>
-      <c r="B352" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -4646,11 +3181,6 @@
           <t>82</t>
         </is>
       </c>
-      <c r="B353" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -4658,11 +3188,6 @@
           <t>83</t>
         </is>
       </c>
-      <c r="B354" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 1C, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -4670,11 +3195,6 @@
           <t>84</t>
         </is>
       </c>
-      <c r="B355" t="inlineStr">
-        <is>
-          <t>1, 10, 2A, 2B, 3A, 3B, 3C, 4, 5, 6, 7A, 7B, 8A, 8B, 8C, 9</t>
-        </is>
-      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -4682,11 +3202,6 @@
           <t>85</t>
         </is>
       </c>
-      <c r="B356" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -4694,11 +3209,6 @@
           <t>86</t>
         </is>
       </c>
-      <c r="B357" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -4706,11 +3216,6 @@
           <t>87</t>
         </is>
       </c>
-      <c r="B358" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -4718,11 +3223,6 @@
           <t>88</t>
         </is>
       </c>
-      <c r="B359" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -4730,11 +3230,6 @@
           <t>89</t>
         </is>
       </c>
-      <c r="B360" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25A, 25B, 25C1, 25C2, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -4742,11 +3237,6 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B361" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -4754,11 +3244,6 @@
           <t>90</t>
         </is>
       </c>
-      <c r="B362" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -4766,11 +3251,6 @@
           <t>91</t>
         </is>
       </c>
-      <c r="B363" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -4778,11 +3258,6 @@
           <t>92</t>
         </is>
       </c>
-      <c r="B364" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -4790,11 +3265,6 @@
           <t>93</t>
         </is>
       </c>
-      <c r="B365" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -4802,11 +3272,6 @@
           <t>94</t>
         </is>
       </c>
-      <c r="B366" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -4814,11 +3279,6 @@
           <t>95</t>
         </is>
       </c>
-      <c r="B367" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 1A, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -4826,11 +3286,6 @@
           <t>96</t>
         </is>
       </c>
-      <c r="B368" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -4838,11 +3293,6 @@
           <t>97</t>
         </is>
       </c>
-      <c r="B369" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16, 17, 18A, 18B, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 5A1A1A1, 5A2, 6A1A1A1, 6A2, 6B, 7B, 8A1A1A, 8A2, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -4850,21 +3300,11 @@
           <t>98</t>
         </is>
       </c>
-      <c r="B370" t="inlineStr">
-        <is>
-          <t>10, 1A1, 1A2, 2, 2A1A1A, 2A2, 2B, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
           <t>99</t>
-        </is>
-      </c>
-      <c r="B371" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>